<commit_message>
feat: add Work Breakdown Structure spreadsheet for procurement management system
</commit_message>
<xml_diff>
--- a/guide/WBS_Procurement_Management_System.xlsx
+++ b/guide/WBS_Procurement_Management_System.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping Requirement" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules &amp; Open Questions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Checklist" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimasi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WBS Detail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mapping Requirement" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Milestone" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rules &amp; Open Questions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Test Checklist" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Estimasi" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Petunjuk'!$A$1:$B$14</definedName>
@@ -900,7 +900,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Perlu finalisasi</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Berjalan</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Perlu dicek</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Berjalan</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Opsional</t>
+          <t>Selesai (dashboard queue)</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Belum mulai</t>
+          <t>Selesai</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Selesaikan deliverable analisis sebelum fitur inti.</t>
+          <t>Selesai. BRD, PRD, BPMN, ERD, rancangan UI terdokumentasi.</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Setup teknis sudah sebagian dilakukan.</t>
+          <t>Selesai. Django+PostgreSQL setup, .env, login/logout, RBAC, Django Admin.</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Prioritas demo tertinggi.</t>
+          <t>Selesai. Form 2-kolom accordion, validasi, approval 5 tahap, matriks nominal, re-approval.</t>
         </is>
       </c>
     </row>
@@ -3892,7 +3892,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Pembayaran dan aplikasi warehouse di luar scope.</t>
+          <t>Selesai. PO creation, print view, penerimaan parsial, discrepancy, penutupan.</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Sederhanakan UI bila waktu terbatas.</t>
+          <t>Selesai. Cancellation request/decide, status restore, AuditEvent trail.</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Estimasi awal.</t>
+          <t>Selesai. 32 unit/integration tests pass, README.md lengkap, seed_dummy_data.</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Kerjakan hanya jika fitur inti selesai.</t>
+          <t>Tidak dikerjakan (opsional, di luar MVP).</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Harga, kualitas, lead time, compliance, atau kriteria lain?</t>
+          <t>4 kriteria: harga, kualitas, lead time, compliance (skor 0-100). Rata-rata sebagai total score.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4409,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Apakah perubahan material membatalkan approval terdahulu? Rekomendasi: review ulang.</t>
+          <t>Ya, perubahan material (nominal/supplier) mereset approval ke Section Head. Evaluasi dihapus.</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Sampai tahap mana requester boleh meminta pembatalan?</t>
+          <t>Pembatalan hanya diizinkan sebelum PO diterbitkan. Setelah PO ada, cancellation ditolak sistem.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Bagaimana mengukur penyelesaian jasa: kuantitas, milestone, atau sign-off?</t>
+          <t>ServiceMilestone per item jasa; milestone ditandai selesai oleh Receiver/Procurement.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>PDF, print view, dan pola nomor PO seperti apa yang dibutuhkan?</t>
+          <t>Print-friendly HTML (po_print.html), nomor PO-YYYYMMDD-UUID, simpan PDF dari browser.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Perlu konfirmasi</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>In-app saja atau email juga?</t>
+          <t>In-app dashboard queue per role. Email opsional, tidak diimplementasikan pada MVP.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Opsional / perlu putuskan</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4670,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (integration test)</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (unit test)</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Belum diuji</t>
+          <t>Lulus (manual)</t>
         </is>
       </c>
     </row>

</xml_diff>